<commit_message>
Update project status and improve HTML structure
</commit_message>
<xml_diff>
--- a/佐賀観光ポートフォリオ_制作管理表_v1.0.xlsx
+++ b/佐賀観光ポートフォリオ_制作管理表_v1.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3dd9ec8ee41f2d3a/デスクトップ/saga-small-trip/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{99242C6B-F4AC-4392-AB20-838993D92F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6336AD6C-694D-4DE4-B9B1-F1BDE8052B92}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{99242C6B-F4AC-4392-AB20-838993D92F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23B81473-D642-4302-9CC0-BEE80157D0FF}"/>
   <bookViews>
-    <workbookView xWindow="1208" yWindow="375" windowWidth="11857" windowHeight="13035" xr2:uid="{EE90897B-71E4-4343-8F25-66AB760EE550}"/>
+    <workbookView xWindow="263" yWindow="293" windowWidth="11047" windowHeight="13034" xr2:uid="{EE90897B-71E4-4343-8F25-66AB760EE550}"/>
   </bookViews>
   <sheets>
     <sheet name="制作進捗" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="60">
   <si>
     <t>佐賀県観光ポートフォリオ制作進捗管理表</t>
     <rPh sb="0" eb="3">
@@ -477,6 +477,16 @@
       <t>コウカイ</t>
     </rPh>
     <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>進行中</t>
+  </si>
+  <si>
+    <t>画像以外の表示確認は完了。残りの画像を準備中。</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>公開テスト完了。制作継続のため現在は一時非公開。</t>
   </si>
 </sst>
 </file>
@@ -1482,7 +1492,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>46280</v>
+        <v>46283</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -1532,14 +1542,14 @@
       </c>
       <c r="D5" s="7">
         <f>COUNTIF(F9:F19,"完了")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>5</v>
       </c>
       <c r="F5" s="8">
         <f>IFERROR(D5/B5,0)</f>
-        <v>0.36363636363636365</v>
+        <v>0.54545454545454541</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -1712,11 +1722,11 @@
       </c>
       <c r="H12" s="11"/>
       <c r="I12" s="2">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="J12" s="12"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="13" spans="1:10" ht="33" x14ac:dyDescent="0.7">
       <c r="A13" s="1">
         <v>5</v>
       </c>
@@ -1733,14 +1743,16 @@
         <v>31</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>35</v>
       </c>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
-      <c r="J13" s="12"/>
+      <c r="J13" s="12" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.7">
       <c r="A14" s="1">
@@ -1759,16 +1771,18 @@
         <v>32</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G14" s="11" t="s">
         <v>35</v>
       </c>
       <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
+      <c r="I14" s="2">
+        <v>46282</v>
+      </c>
       <c r="J14" s="12"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="15" spans="1:10" ht="33" x14ac:dyDescent="0.7">
       <c r="A15" s="1">
         <v>7</v>
       </c>
@@ -1785,14 +1799,18 @@
         <v>56</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G15" s="11" t="s">
         <v>35</v>
       </c>
       <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="12"/>
+      <c r="I15" s="2">
+        <v>46282</v>
+      </c>
+      <c r="J15" s="12" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.7">
       <c r="A16" s="1">

</xml_diff>

<commit_message>
Update project progress after JavaScript features
</commit_message>
<xml_diff>
--- a/佐賀観光ポートフォリオ_制作管理表_v1.0.xlsx
+++ b/佐賀観光ポートフォリオ_制作管理表_v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3dd9ec8ee41f2d3a/デスクトップ/saga-small-trip/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="8_{99242C6B-F4AC-4392-AB20-838993D92F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23B81473-D642-4302-9CC0-BEE80157D0FF}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{99242C6B-F4AC-4392-AB20-838993D92F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B783D1B-375C-471E-8F8C-4BB3960C3F66}"/>
   <bookViews>
     <workbookView xWindow="263" yWindow="293" windowWidth="11047" windowHeight="13034" xr2:uid="{EE90897B-71E4-4343-8F25-66AB760EE550}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="61">
   <si>
     <t>佐賀県観光ポートフォリオ制作進捗管理表</t>
     <rPh sb="0" eb="3">
@@ -286,22 +286,6 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>HTML、CSS、画像を含めてサイト全体を確認する</t>
-    <rPh sb="9" eb="11">
-      <t>ガゾウ</t>
-    </rPh>
-    <rPh sb="12" eb="13">
-      <t>フク</t>
-    </rPh>
-    <rPh sb="18" eb="20">
-      <t>ゼンタイ</t>
-    </rPh>
-    <rPh sb="21" eb="23">
-      <t>カクニン</t>
-    </rPh>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>Git・GitHubの基本を学ぶ</t>
     <rPh sb="11" eb="13">
       <t>キホン</t>
@@ -482,11 +466,31 @@
     <t>進行中</t>
   </si>
   <si>
-    <t>画像以外の表示確認は完了。残りの画像を準備中。</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>公開テスト完了。制作継続のため現在は一時非公開。</t>
+  </si>
+  <si>
+    <t>ハンバーガーメニュー、ページ上部へ戻る、スクロール表示、見どころ絞り込み、グルメ検索を実装。その他の機能追加は後日再開予定。</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>HTML、CSS、JavaScript、画像を含めてサイト全体を確認する</t>
+    <rPh sb="20" eb="22">
+      <t>ガゾウ</t>
+    </rPh>
+    <rPh sb="23" eb="24">
+      <t>フク</t>
+    </rPh>
+    <rPh sb="29" eb="31">
+      <t>ゼンタイ</t>
+    </rPh>
+    <rPh sb="32" eb="34">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>HTML、CSS、JavaScriptの表示・動作確認は完了。残りの画像を準備中。</t>
+    <phoneticPr fontId="2"/>
   </si>
 </sst>
 </file>
@@ -1542,14 +1546,14 @@
       </c>
       <c r="D5" s="7">
         <f>COUNTIF(F9:F19,"完了")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>5</v>
       </c>
       <c r="F5" s="8">
         <f>IFERROR(D5/B5,0)</f>
-        <v>0.54545454545454541</v>
+        <v>0.63636363636363635</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -1631,10 +1635,10 @@
         <v>27</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H9" s="11"/>
       <c r="I9" s="2">
@@ -1659,10 +1663,10 @@
         <v>28</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H10" s="11"/>
       <c r="I10" s="2">
@@ -1687,10 +1691,10 @@
         <v>29</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H11" s="11"/>
       <c r="I11" s="2">
@@ -1715,10 +1719,10 @@
         <v>30</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H12" s="11"/>
       <c r="I12" s="2">
@@ -1726,7 +1730,7 @@
       </c>
       <c r="J12" s="12"/>
     </row>
-    <row r="13" spans="1:10" ht="33" x14ac:dyDescent="0.7">
+    <row r="13" spans="1:10" ht="49.5" x14ac:dyDescent="0.7">
       <c r="A13" s="1">
         <v>5</v>
       </c>
@@ -1737,21 +1741,21 @@
         <v>23</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
       <c r="J13" s="12" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.7">
@@ -1768,13 +1772,13 @@
         <v>26</v>
       </c>
       <c r="E14" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="F14" s="11" t="s">
-        <v>33</v>
-      </c>
       <c r="G14" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H14" s="11"/>
       <c r="I14" s="2">
@@ -1796,20 +1800,20 @@
         <v>26</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H15" s="11"/>
       <c r="I15" s="2">
         <v>46282</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.7">
@@ -1820,25 +1824,25 @@
         <v>18</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D16" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="12" t="s">
-        <v>41</v>
-      </c>
       <c r="F16" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
       <c r="J16" s="12"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="17" spans="1:10" ht="82.5" x14ac:dyDescent="0.7">
       <c r="A17" s="1">
         <v>9</v>
       </c>
@@ -1846,23 +1850,27 @@
         <v>18</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="12"/>
+      <c r="I17" s="2">
+        <v>46285</v>
+      </c>
+      <c r="J17" s="12" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.7">
       <c r="A18" s="1">
@@ -1872,19 +1880,19 @@
         <v>18</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H18" s="11"/>
       <c r="I18" s="11"/>
@@ -1898,19 +1906,19 @@
         <v>18</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>26</v>
       </c>
       <c r="E19" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="11" t="s">
         <v>44</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>45</v>
       </c>
       <c r="H19" s="11"/>
       <c r="I19" s="11"/>
@@ -1959,7 +1967,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="25.9" x14ac:dyDescent="0.7">
       <c r="A1" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.7">
@@ -1972,7 +1980,7 @@
     </row>
     <row r="4" spans="1:11" ht="19.899999999999999" x14ac:dyDescent="0.7">
       <c r="A4" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.7">
@@ -1983,28 +1991,28 @@
         <v>10</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="E5" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="G5" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="9" t="s">
         <v>54</v>
-      </c>
-      <c r="J5" s="9" t="s">
-        <v>55</v>
       </c>
       <c r="K5" s="9" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
Update image asset management sheet
</commit_message>
<xml_diff>
--- a/佐賀観光ポートフォリオ_制作管理表_v1.0.xlsx
+++ b/佐賀観光ポートフォリオ_制作管理表_v1.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3dd9ec8ee41f2d3a/デスクトップ/saga-small-trip/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{99242C6B-F4AC-4392-AB20-838993D92F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B783D1B-375C-471E-8F8C-4BB3960C3F66}"/>
+  <xr:revisionPtr revIDLastSave="430" documentId="8_{99242C6B-F4AC-4392-AB20-838993D92F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71ABEB53-913E-4025-8EE4-9D730DF5AF42}"/>
   <bookViews>
-    <workbookView xWindow="263" yWindow="293" windowWidth="11047" windowHeight="13034" xr2:uid="{EE90897B-71E4-4343-8F25-66AB760EE550}"/>
+    <workbookView xWindow="263" yWindow="293" windowWidth="11047" windowHeight="13320" activeTab="1" xr2:uid="{EE90897B-71E4-4343-8F25-66AB760EE550}"/>
   </bookViews>
   <sheets>
     <sheet name="制作進捗" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="169">
   <si>
     <t>佐賀県観光ポートフォリオ制作進捗管理表</t>
     <rPh sb="0" eb="3">
@@ -491,6 +491,614 @@
   <si>
     <t>HTML、CSS、JavaScriptの表示・動作確認は完了。残りの画像を準備中。</t>
     <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>トップページ</t>
+  </si>
+  <si>
+    <t>画像</t>
+  </si>
+  <si>
+    <t>imarin-beach.JPG</t>
+  </si>
+  <si>
+    <t>イマリンビーチ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>準備済み</t>
+  </si>
+  <si>
+    <t>未加工</t>
+  </si>
+  <si>
+    <t>掲載済み</t>
+  </si>
+  <si>
+    <t>ぱくたそ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>imari-river.JPG</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>伊万里川</t>
+    <rPh sb="0" eb="4">
+      <t>イマリガワ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>okawachiyama.JPG</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>大川内山</t>
+    <rPh sb="0" eb="4">
+      <t>オオカワウチヤマ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>未掲載</t>
+  </si>
+  <si>
+    <t>モデルコース</t>
+  </si>
+  <si>
+    <t>画像</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>yobuko-squid.JPG</t>
+  </si>
+  <si>
+    <t>呼子のイカ</t>
+    <rPh sb="0" eb="2">
+      <t>ヨブコ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>saga-beef.JPG</t>
+  </si>
+  <si>
+    <t>ureshino-onsen-yudofu.JPG</t>
+  </si>
+  <si>
+    <t>佐賀牛</t>
+    <rPh sb="0" eb="3">
+      <t>サガギュウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>嬉野温泉湯どうふ</t>
+    <rPh sb="0" eb="4">
+      <t>ウレシノオンセン</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>ユ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ureshino-siebold-bath.JPG</t>
+  </si>
+  <si>
+    <t>嬉野温泉・シーボルトの湯</t>
+    <rPh sb="0" eb="2">
+      <t>ウレシノ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>オンセン</t>
+    </rPh>
+    <rPh sb="11" eb="12">
+      <t>ユ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ureshino-onsen-street.JPG</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ureshino-siebold-footbath.JPG</t>
+  </si>
+  <si>
+    <t>嬉野温泉街</t>
+    <rPh sb="0" eb="2">
+      <t>ウレシノ</t>
+    </rPh>
+    <rPh sb="2" eb="5">
+      <t>オンセンガイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>嬉野温泉・シーボルトのあし湯</t>
+    <rPh sb="0" eb="4">
+      <t>ウレシノオンセン</t>
+    </rPh>
+    <rPh sb="13" eb="14">
+      <t>ユ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>okawachiyama-street.JPG</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>aioi-bridge.JPG</t>
+  </si>
+  <si>
+    <t>koimari-park.JPG</t>
+  </si>
+  <si>
+    <t>大川内山・石畳の街並み</t>
+    <rPh sb="0" eb="4">
+      <t>オオカワウチヤマ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>イシダタミ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>マチナ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>相生橋</t>
+    <rPh sb="0" eb="3">
+      <t>アイオイバシ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>古伊万里公園</t>
+    <rPh sb="0" eb="6">
+      <t>コイマリコウエン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>準備中</t>
+  </si>
+  <si>
+    <t>タイル型メニュー・SNS画像・コース内スポット</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>コース内スポット</t>
+    <rPh sb="3" eb="4">
+      <t>ナイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ureshino-onsen-aerial.JPG</t>
+  </si>
+  <si>
+    <t>旅の締めくくり</t>
+    <rPh sb="0" eb="1">
+      <t>タビ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>シ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>takeo-onsen-station.JPG</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>hamanoura-terraced-fields-sunset.JPG</t>
+  </si>
+  <si>
+    <t>武雄温泉駅</t>
+    <rPh sb="0" eb="5">
+      <t>タケオオンセンエキ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>浜野浦の棚田の夕日</t>
+    <rPh sb="0" eb="3">
+      <t>ハマノウラ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>タナダ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>ユウヒ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タイル型メニュー・SNS画像・見どころカード</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タイル型メニュー・コース内スポット・おすすめ・見どころカード</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>TOPページ内で2か所と見どころページでも使用</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>モデルコース・見どころページでも使用</t>
+    <rPh sb="7" eb="8">
+      <t>ミ</t>
+    </rPh>
+    <rPh sb="16" eb="18">
+      <t>シヨウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>見どころページでも使用</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>佐賀の見どころ</t>
+  </si>
+  <si>
+    <t>見どころカード</t>
+    <rPh sb="0" eb="1">
+      <t>ミ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>nagoya-castle.JPG</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>名護屋城跡</t>
+    <rPh sb="0" eb="5">
+      <t>ナゴヤジョウアト</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>saga-castle-honmaru-history-museum.JPG</t>
+  </si>
+  <si>
+    <t>taku-seibyo.JPG</t>
+  </si>
+  <si>
+    <t>karatsu-castle-town.JPG</t>
+  </si>
+  <si>
+    <t>佐賀城本丸歴史館</t>
+    <rPh sb="0" eb="8">
+      <t>サガジョウホンマルレキシカン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>多久聖廟</t>
+    <rPh sb="0" eb="4">
+      <t>タクセイビョウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>唐津城下町</t>
+    <rPh sb="0" eb="5">
+      <t>カラツジョウカマチ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>yoshinogari-historical-park.JPG</t>
+  </si>
+  <si>
+    <t>tozan-shrine.JPG</t>
+  </si>
+  <si>
+    <t>niji-no-matsubara.JPG</t>
+  </si>
+  <si>
+    <t>吉野ヶ里歴史公園</t>
+    <rPh sb="0" eb="8">
+      <t>ヨシノガリレキシコウエン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>陶山神社</t>
+    <rPh sb="0" eb="4">
+      <t>スエヤマジンジャ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>虹の松原</t>
+    <rPh sb="0" eb="1">
+      <t>ニジ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>マツバラ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タイル型メニュー・SNS画像・グルメカード</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タイル型メニュー・コース内スポット・グルメカード</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>TOPページ内で2か所とグルメページでも使用</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>モデルコース・グルメページでも使用</t>
+    <rPh sb="15" eb="17">
+      <t>シヨウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>グルメ</t>
+  </si>
+  <si>
+    <t>グルメ紹介</t>
+    <rPh sb="3" eb="5">
+      <t>ショウカイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>未加工</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>sicilian-rice.JPG</t>
+  </si>
+  <si>
+    <t>シシリアンライス</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>takezaki-crab.JPG</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>竹崎カニ</t>
+    <rPh sb="0" eb="2">
+      <t>タケサキ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>saga-ramen.JPG</t>
+  </si>
+  <si>
+    <t>佐賀ラーメン</t>
+    <rPh sb="0" eb="2">
+      <t>サガ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>marubouro.JPG</t>
+  </si>
+  <si>
+    <t>丸ぼうろ</t>
+    <rPh sb="0" eb="1">
+      <t>マル</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>温泉</t>
+  </si>
+  <si>
+    <t>温泉紹介カード</t>
+    <rPh sb="0" eb="4">
+      <t>オンセンショウカイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>takeo-onsen.JPG</t>
+  </si>
+  <si>
+    <t>furuyu-onsen.JPG</t>
+  </si>
+  <si>
+    <t>古湯温泉</t>
+    <rPh sb="0" eb="2">
+      <t>フルユ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>オンセン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>chikugo-river-lift-bridge.JPG</t>
+  </si>
+  <si>
+    <t>筑後川昇開橋</t>
+    <rPh sb="0" eb="3">
+      <t>チクゴガワ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ショウカイ</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>バシ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>About</t>
+  </si>
+  <si>
+    <t>コンセプト画像</t>
+    <rPh sb="5" eb="7">
+      <t>ガゾウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>yutoku-inari-shrine.JPG</t>
+  </si>
+  <si>
+    <t>佐賀平野を飛ぶバルーン</t>
+    <rPh sb="0" eb="4">
+      <t>サガヘイヤ</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>ト</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>祐徳稲荷神社</t>
+    <rPh sb="0" eb="6">
+      <t>ユウトクイナリジンジャ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>画像を準備中</t>
+    <rPh sb="0" eb="2">
+      <t>ガゾウ</t>
+    </rPh>
+    <rPh sb="3" eb="6">
+      <t>ジュンビチュウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>使用場所を検討中</t>
+    <rPh sb="0" eb="4">
+      <t>シヨウバショ</t>
+    </rPh>
+    <rPh sb="5" eb="8">
+      <t>ケントウチュウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>gyoza-kaikan.JPG</t>
+  </si>
+  <si>
+    <t>餃子会館</t>
+    <rPh sb="0" eb="4">
+      <t>ギョウザカイカン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>掲載保留中</t>
+    <rPh sb="0" eb="5">
+      <t>ケイサイホリュウチュウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タイル型メニュー</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タイル型メニュー</t>
+    <rPh sb="3" eb="4">
+      <t>ガタ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タイル型メニュー・見どころカード</t>
+    <rPh sb="9" eb="10">
+      <t>ミ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タイル型メニュー・おすすめ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>タイル型メニュー</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>モデルコース用タイル</t>
+    <rPh sb="6" eb="7">
+      <t>ヨウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>TOPページ内で2か所、モデルコース・温泉ページでも使用</t>
+    <rPh sb="6" eb="7">
+      <t>ナイ</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>ショ</t>
+    </rPh>
+    <rPh sb="19" eb="21">
+      <t>オンセン</t>
+    </rPh>
+    <rPh sb="26" eb="28">
+      <t>シヨウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>モデルコースでも使用</t>
+    <rPh sb="8" eb="10">
+      <t>シヨウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>嬉野温泉街　上空</t>
+    <rPh sb="0" eb="4">
+      <t>ウレシノオンセン</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>ガイ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ジョウクウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>武雄温泉</t>
+    <rPh sb="0" eb="4">
+      <t>タケオオンセン</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>saga-balloon.JPG</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>サイト紹介画像</t>
+    <rPh sb="3" eb="5">
+      <t>ショウカイ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ガゾウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>photoAC</t>
   </si>
 </sst>
 </file>
@@ -500,7 +1108,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -567,6 +1175,12 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -599,7 +1213,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -639,12 +1253,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="パーセント" xfId="1" builtinId="5"/>
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="33">
+  <dxfs count="31">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -724,179 +1347,6 @@
           <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1092,6 +1542,147 @@
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -1126,41 +1717,39 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{45746EF6-A68A-45AA-AB1C-9DEFD8F177FB}" name="テーブル1" displayName="テーブル1" ref="A8:J19" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{45746EF6-A68A-45AA-AB1C-9DEFD8F177FB}" name="テーブル1" displayName="テーブル1" ref="A8:J19" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="A8:J19" xr:uid="{45746EF6-A68A-45AA-AB1C-9DEFD8F177FB}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{0FC2ED50-DED0-452D-8651-DFEEA5362CCC}" name="No." dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{B004CBA6-95FD-4E4A-A3E6-402761BF9C72}" name="公開段階　" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{FCE9EC5D-92C5-4A3D-9681-1FB0E660864E}" name="分類" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{E7F1C059-5D29-4EBF-9210-A2C29E8D3479}" name="対象ページ" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{1B503DAA-F560-4720-9589-DF77055BC3C2}" name="作業内容" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{79045720-24B4-4F4A-A27C-E7EA47907295}" name="状況" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{C5197FD5-F06F-4FC6-8A53-3CF7D71D9B4B}" name="優先度" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{BF7CAD6E-7D39-4261-B83D-B6D0E5FED90F}" name="期限" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{82358B19-5A5A-4B33-9E26-92CF4591F4F3}" name="完了日" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{5350E184-4ED2-466B-9154-DD78A175EF90}" name="備考" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{0FC2ED50-DED0-452D-8651-DFEEA5362CCC}" name="No." dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{B004CBA6-95FD-4E4A-A3E6-402761BF9C72}" name="公開段階　" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{FCE9EC5D-92C5-4A3D-9681-1FB0E660864E}" name="分類" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{E7F1C059-5D29-4EBF-9210-A2C29E8D3479}" name="対象ページ" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{1B503DAA-F560-4720-9589-DF77055BC3C2}" name="作業内容" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{79045720-24B4-4F4A-A27C-E7EA47907295}" name="状況" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{C5197FD5-F06F-4FC6-8A53-3CF7D71D9B4B}" name="優先度" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{BF7CAD6E-7D39-4261-B83D-B6D0E5FED90F}" name="期限" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{82358B19-5A5A-4B33-9E26-92CF4591F4F3}" name="完了日" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{5350E184-4ED2-466B-9154-DD78A175EF90}" name="備考" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{546C232F-F352-4C04-8BE9-61C2F77D47FF}" name="テーブル2" displayName="テーブル2" ref="A5:K6" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
-  <autoFilter ref="A5:K6" xr:uid="{546C232F-F352-4C04-8BE9-61C2F77D47FF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{546C232F-F352-4C04-8BE9-61C2F77D47FF}" name="テーブル2" displayName="テーブル2" ref="A5:K37" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
+  <autoFilter ref="A5:K37" xr:uid="{546C232F-F352-4C04-8BE9-61C2F77D47FF}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{3AFE5A2E-5BD4-41A6-B804-8B249DFE51BF}" name="No." dataDxfId="18">
-      <calculatedColumnFormula>IF(B6="","",ROW()-5)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{BB467987-83AD-4E6C-94CE-359A061C2269}" name="対象ページ" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{91BA6E35-CF34-44CE-A1CD-924D988B374F}" name="使用場所" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{1284F502-B299-4748-9A33-EEF78A96B113}" name="素材種別" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{AE73E1C8-AD9C-41F2-B73D-E524973D4844}" name="ファイル名" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{5F6BCA63-3B29-42F8-A5BF-B347F5CF904A}" name="素材内容" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{99925BCF-9D8B-4300-BF92-966364F1E7F8}" name="準備状況" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{B38E0B3B-668D-4DFF-BCEA-20D28022E34A}" name="加工状況" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{DB88FA17-092A-49F9-A686-A3FE1483036F}" name="掲載状況" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{613559A8-2FBF-4036-A4FF-18B4B1B3E2E8}" name="出典・入手先" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{1C562C7E-EF5E-4300-B623-7ECCBAD59A8B}" name="備考" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{3AFE5A2E-5BD4-41A6-B804-8B249DFE51BF}" name="No." dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{BB467987-83AD-4E6C-94CE-359A061C2269}" name="対象ページ" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{91BA6E35-CF34-44CE-A1CD-924D988B374F}" name="使用場所"/>
+    <tableColumn id="4" xr3:uid="{1284F502-B299-4748-9A33-EEF78A96B113}" name="素材種別" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{AE73E1C8-AD9C-41F2-B73D-E524973D4844}" name="ファイル名"/>
+    <tableColumn id="6" xr3:uid="{5F6BCA63-3B29-42F8-A5BF-B347F5CF904A}" name="素材内容" dataDxfId="25"/>
+    <tableColumn id="7" xr3:uid="{99925BCF-9D8B-4300-BF92-966364F1E7F8}" name="準備状況" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{B38E0B3B-668D-4DFF-BCEA-20D28022E34A}" name="加工状況" dataDxfId="23"/>
+    <tableColumn id="9" xr3:uid="{DB88FA17-092A-49F9-A686-A3FE1483036F}" name="掲載状況" dataDxfId="22"/>
+    <tableColumn id="10" xr3:uid="{613559A8-2FBF-4036-A4FF-18B4B1B3E2E8}" name="出典・入手先" dataDxfId="21"/>
+    <tableColumn id="11" xr3:uid="{1C562C7E-EF5E-4300-B623-7ECCBAD59A8B}" name="備考" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1464,7 +2053,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2652F556-56E9-49EB-9323-CCD84DCD67E1}">
   <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="6.5625" customWidth="1"/>
     <col min="2" max="2" width="12.5625" customWidth="1"/>
@@ -1477,7 +2066,7 @@
     <col min="10" max="10" width="25.5625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="25.9" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:10" ht="25.9">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1491,7 +2080,7 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1507,7 +2096,7 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:10">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1519,7 +2108,7 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:10" ht="19.899999999999999" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:10" ht="19.899999999999999">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -1533,7 +2122,7 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:10" ht="19.899999999999999" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:10" ht="19.899999999999999">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
@@ -1560,7 +2149,7 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:10">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1572,7 +2161,7 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:10">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1586,7 +2175,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:10">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -1618,7 +2207,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:10">
       <c r="A9" s="1">
         <v>1</v>
       </c>
@@ -1646,7 +2235,7 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:10">
       <c r="A10" s="1">
         <v>2</v>
       </c>
@@ -1674,7 +2263,7 @@
       </c>
       <c r="J10" s="12"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="11" spans="1:10">
       <c r="A11" s="1">
         <v>3</v>
       </c>
@@ -1702,7 +2291,7 @@
       </c>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="12" spans="1:10">
       <c r="A12" s="1">
         <v>4</v>
       </c>
@@ -1730,7 +2319,7 @@
       </c>
       <c r="J12" s="12"/>
     </row>
-    <row r="13" spans="1:10" ht="49.5" x14ac:dyDescent="0.7">
+    <row r="13" spans="1:10" ht="49.5">
       <c r="A13" s="1">
         <v>5</v>
       </c>
@@ -1758,7 +2347,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="14" spans="1:10">
       <c r="A14" s="1">
         <v>6</v>
       </c>
@@ -1786,7 +2375,7 @@
       </c>
       <c r="J14" s="12"/>
     </row>
-    <row r="15" spans="1:10" ht="33" x14ac:dyDescent="0.7">
+    <row r="15" spans="1:10" ht="33">
       <c r="A15" s="1">
         <v>7</v>
       </c>
@@ -1816,7 +2405,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="16" spans="1:10">
       <c r="A16" s="1">
         <v>8</v>
       </c>
@@ -1842,7 +2431,7 @@
       <c r="I16" s="11"/>
       <c r="J16" s="12"/>
     </row>
-    <row r="17" spans="1:10" ht="82.5" x14ac:dyDescent="0.7">
+    <row r="17" spans="1:10" ht="82.5">
       <c r="A17" s="1">
         <v>9</v>
       </c>
@@ -1872,7 +2461,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.7">
+    <row r="18" spans="1:10">
       <c r="A18" s="1">
         <v>10</v>
       </c>
@@ -1898,7 +2487,7 @@
       <c r="I18" s="11"/>
       <c r="J18" s="12"/>
     </row>
-    <row r="19" spans="1:10" ht="33" x14ac:dyDescent="0.7">
+    <row r="19" spans="1:10" ht="33">
       <c r="A19" s="1">
         <v>11</v>
       </c>
@@ -1952,7 +2541,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2B46C85-171F-4A6A-84E0-A39E9DFB6A75}">
   <dimension ref="A1:K100"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="6.5625" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.5625" style="1" customWidth="1"/>
@@ -1965,25 +2554,25 @@
     <col min="12" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="25.9" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:11" ht="25.9">
       <c r="A1" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:11">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>46280</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="19.899999999999999" x14ac:dyDescent="0.7">
+        <v>46285</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="19.899999999999999">
       <c r="A4" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:11">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -2018,330 +2607,1097 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A6" s="10" t="str">
-        <f>IF(B6="","",ROW()-5)</f>
-        <v/>
-      </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A21" s="10"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="9"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A24" s="10"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A25" s="10"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="J25" s="9"/>
-      <c r="K25" s="9"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="J26" s="9"/>
-      <c r="K26" s="9"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="9"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="J28" s="9"/>
-      <c r="K28" s="9"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A29" s="10"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="J29" s="9"/>
-      <c r="K29" s="9"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="J30" s="9"/>
-      <c r="K30" s="9"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="9"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="J32" s="9"/>
-      <c r="K32" s="9"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="J33" s="9"/>
-      <c r="K33" s="9"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="J34" s="9"/>
-      <c r="K34" s="9"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="J35" s="9"/>
-      <c r="K35" s="9"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="J36" s="9"/>
-      <c r="K36" s="9"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.7">
-      <c r="A37" s="10"/>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="J37" s="9"/>
-      <c r="K37" s="9"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:11" ht="33">
+      <c r="A6" s="10">
+        <v>1</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="K6" s="9" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="33">
+      <c r="A7" s="13">
+        <v>2</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="33">
+      <c r="A8" s="13">
+        <v>3</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="K8" s="12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="33">
+      <c r="A9" s="13">
+        <v>4</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K9" s="12" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="33">
+      <c r="A10" s="13">
+        <v>5</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J10" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="33">
+      <c r="A11" s="13">
+        <v>6</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E11" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J11" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="33">
+      <c r="A12" s="13">
+        <v>7</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" t="s">
+        <v>82</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="17.649999999999999">
+      <c r="A13" s="13">
+        <v>8</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J13" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K13" s="14" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="17.649999999999999">
+      <c r="A14" s="13">
+        <v>9</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E14" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J14" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K14" s="15"/>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="13">
+        <v>10</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J15" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="K15" s="12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="17.649999999999999">
+      <c r="A16" s="13">
+        <v>11</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" t="s">
+        <v>89</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J16" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="K16" s="12" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="17.649999999999999">
+      <c r="A17" s="13">
+        <v>12</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J17" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="K17" s="12"/>
+    </row>
+    <row r="18" spans="1:11" ht="17.649999999999999">
+      <c r="A18" s="13">
+        <v>13</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E18" t="s">
+        <v>144</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K18" s="12" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="17.649999999999999">
+      <c r="A19" s="13">
+        <v>14</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" t="s">
+        <v>97</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J19" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K19" s="12"/>
+    </row>
+    <row r="20" spans="1:11" ht="17.649999999999999">
+      <c r="A20" s="13">
+        <v>15</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" t="s">
+        <v>99</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K20" s="12" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="17.649999999999999">
+      <c r="A21" s="13">
+        <v>16</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" t="s">
+        <v>100</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I21" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="J21" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K21" s="12" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" s="13">
+        <v>17</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K22" s="12"/>
+    </row>
+    <row r="23" spans="1:11" ht="17.649999999999999">
+      <c r="A23" s="13">
+        <v>18</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" t="s">
+        <v>112</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I23" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J23" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K23" s="12"/>
+    </row>
+    <row r="24" spans="1:11" ht="17.649999999999999">
+      <c r="A24" s="13">
+        <v>19</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E24" t="s">
+        <v>113</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K24" s="12"/>
+    </row>
+    <row r="25" spans="1:11" ht="17.649999999999999">
+      <c r="A25" s="13">
+        <v>20</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="G25" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I25" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J25" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K25" s="12"/>
+    </row>
+    <row r="26" spans="1:11" ht="17.649999999999999">
+      <c r="A26" s="13">
+        <v>21</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E26" t="s">
+        <v>118</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H26" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I26" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K26" s="12"/>
+    </row>
+    <row r="27" spans="1:11" ht="17.649999999999999">
+      <c r="A27" s="13">
+        <v>22</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" t="s">
+        <v>119</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H27" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I27" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J27" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K27" s="12"/>
+    </row>
+    <row r="28" spans="1:11" ht="17.649999999999999">
+      <c r="A28" s="13">
+        <v>23</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E28" t="s">
+        <v>120</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K28" s="12"/>
+    </row>
+    <row r="29" spans="1:11" ht="17.649999999999999">
+      <c r="A29" s="13">
+        <v>24</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" t="s">
+        <v>131</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H29" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J29" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K29" s="12"/>
+    </row>
+    <row r="30" spans="1:11">
+      <c r="A30" s="13">
+        <v>25</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J30" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K30" s="12"/>
+    </row>
+    <row r="31" spans="1:11" ht="17.649999999999999">
+      <c r="A31" s="13">
+        <v>26</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E31" t="s">
+        <v>135</v>
+      </c>
+      <c r="F31" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="J31" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K31" s="12" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="17.649999999999999">
+      <c r="A32" s="13">
+        <v>27</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E32" t="s">
+        <v>137</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="G32" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K32" s="12"/>
+    </row>
+    <row r="33" spans="1:11" ht="17.649999999999999">
+      <c r="A33" s="13">
+        <v>28</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E33" t="s">
+        <v>141</v>
+      </c>
+      <c r="F33" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J33" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K33" s="12"/>
+    </row>
+    <row r="34" spans="1:11" ht="17.649999999999999">
+      <c r="A34" s="13">
+        <v>29</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E34" t="s">
+        <v>142</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="G34" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I34" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J34" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K34" s="12"/>
+    </row>
+    <row r="35" spans="1:11" ht="17.649999999999999">
+      <c r="A35" s="13">
+        <v>30</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E35" t="s">
+        <v>166</v>
+      </c>
+      <c r="F35" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="G35" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="H35" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I35" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="J35" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K35" s="12" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="17.649999999999999">
+      <c r="A36" s="13">
+        <v>31</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E36" t="s">
+        <v>148</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="G36" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="H36" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I36" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="J36" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K36" s="12" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="17.649999999999999">
+      <c r="A37" s="13">
+        <v>32</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E37" t="s">
+        <v>153</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="G37" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H37" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I37" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="J37" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="K37" s="12" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
       <c r="A38" s="10"/>
       <c r="B38" s="10"/>
       <c r="C38" s="10"/>
@@ -2351,7 +3707,7 @@
       <c r="J38" s="9"/>
       <c r="K38" s="9"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="39" spans="1:11">
       <c r="A39" s="10"/>
       <c r="B39" s="10"/>
       <c r="C39" s="10"/>
@@ -2361,7 +3717,7 @@
       <c r="J39" s="9"/>
       <c r="K39" s="9"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="40" spans="1:11">
       <c r="A40" s="10"/>
       <c r="B40" s="10"/>
       <c r="C40" s="10"/>
@@ -2371,7 +3727,7 @@
       <c r="J40" s="9"/>
       <c r="K40" s="9"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="41" spans="1:11">
       <c r="A41" s="10"/>
       <c r="B41" s="10"/>
       <c r="C41" s="10"/>
@@ -2381,7 +3737,7 @@
       <c r="J41" s="9"/>
       <c r="K41" s="9"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="42" spans="1:11">
       <c r="A42" s="10"/>
       <c r="B42" s="10"/>
       <c r="C42" s="10"/>
@@ -2391,7 +3747,7 @@
       <c r="J42" s="9"/>
       <c r="K42" s="9"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="43" spans="1:11">
       <c r="A43" s="10"/>
       <c r="B43" s="10"/>
       <c r="C43" s="10"/>
@@ -2401,7 +3757,7 @@
       <c r="J43" s="9"/>
       <c r="K43" s="9"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="44" spans="1:11">
       <c r="A44" s="10"/>
       <c r="B44" s="10"/>
       <c r="C44" s="10"/>
@@ -2411,7 +3767,7 @@
       <c r="J44" s="9"/>
       <c r="K44" s="9"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="45" spans="1:11">
       <c r="A45" s="10"/>
       <c r="B45" s="10"/>
       <c r="C45" s="10"/>
@@ -2421,7 +3777,7 @@
       <c r="J45" s="9"/>
       <c r="K45" s="9"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="46" spans="1:11">
       <c r="A46" s="10"/>
       <c r="B46" s="10"/>
       <c r="C46" s="10"/>
@@ -2431,7 +3787,7 @@
       <c r="J46" s="9"/>
       <c r="K46" s="9"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="47" spans="1:11">
       <c r="A47" s="10"/>
       <c r="B47" s="10"/>
       <c r="C47" s="10"/>
@@ -2441,7 +3797,7 @@
       <c r="J47" s="9"/>
       <c r="K47" s="9"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="48" spans="1:11">
       <c r="A48" s="10"/>
       <c r="B48" s="10"/>
       <c r="C48" s="10"/>
@@ -2451,7 +3807,7 @@
       <c r="J48" s="9"/>
       <c r="K48" s="9"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="49" spans="1:11">
       <c r="A49" s="10"/>
       <c r="B49" s="10"/>
       <c r="C49" s="10"/>
@@ -2461,7 +3817,7 @@
       <c r="J49" s="9"/>
       <c r="K49" s="9"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="50" spans="1:11">
       <c r="A50" s="10"/>
       <c r="B50" s="10"/>
       <c r="C50" s="10"/>
@@ -2471,7 +3827,7 @@
       <c r="J50" s="9"/>
       <c r="K50" s="9"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="51" spans="1:11">
       <c r="A51" s="10"/>
       <c r="B51" s="10"/>
       <c r="C51" s="10"/>
@@ -2481,7 +3837,7 @@
       <c r="J51" s="9"/>
       <c r="K51" s="9"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="52" spans="1:11">
       <c r="A52" s="10"/>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
@@ -2491,7 +3847,7 @@
       <c r="J52" s="9"/>
       <c r="K52" s="9"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="53" spans="1:11">
       <c r="A53" s="10"/>
       <c r="B53" s="10"/>
       <c r="C53" s="10"/>
@@ -2501,7 +3857,7 @@
       <c r="J53" s="9"/>
       <c r="K53" s="9"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="54" spans="1:11">
       <c r="A54" s="10"/>
       <c r="B54" s="10"/>
       <c r="C54" s="10"/>
@@ -2511,7 +3867,7 @@
       <c r="J54" s="9"/>
       <c r="K54" s="9"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="55" spans="1:11">
       <c r="A55" s="10"/>
       <c r="B55" s="10"/>
       <c r="C55" s="10"/>
@@ -2521,7 +3877,7 @@
       <c r="J55" s="9"/>
       <c r="K55" s="9"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="56" spans="1:11">
       <c r="A56" s="10"/>
       <c r="B56" s="10"/>
       <c r="C56" s="10"/>
@@ -2531,7 +3887,7 @@
       <c r="J56" s="9"/>
       <c r="K56" s="9"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="57" spans="1:11">
       <c r="A57" s="10"/>
       <c r="B57" s="10"/>
       <c r="C57" s="10"/>
@@ -2541,7 +3897,7 @@
       <c r="J57" s="9"/>
       <c r="K57" s="9"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="58" spans="1:11">
       <c r="A58" s="10"/>
       <c r="B58" s="10"/>
       <c r="C58" s="10"/>
@@ -2551,7 +3907,7 @@
       <c r="J58" s="9"/>
       <c r="K58" s="9"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="59" spans="1:11">
       <c r="A59" s="10"/>
       <c r="B59" s="10"/>
       <c r="C59" s="10"/>
@@ -2561,7 +3917,7 @@
       <c r="J59" s="9"/>
       <c r="K59" s="9"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="60" spans="1:11">
       <c r="A60" s="10"/>
       <c r="B60" s="10"/>
       <c r="C60" s="10"/>
@@ -2571,7 +3927,7 @@
       <c r="J60" s="9"/>
       <c r="K60" s="9"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="61" spans="1:11">
       <c r="A61" s="10"/>
       <c r="B61" s="10"/>
       <c r="C61" s="10"/>
@@ -2581,7 +3937,7 @@
       <c r="J61" s="9"/>
       <c r="K61" s="9"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="62" spans="1:11">
       <c r="A62" s="10"/>
       <c r="B62" s="10"/>
       <c r="C62" s="10"/>
@@ -2591,7 +3947,7 @@
       <c r="J62" s="9"/>
       <c r="K62" s="9"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="63" spans="1:11">
       <c r="A63" s="10"/>
       <c r="B63" s="10"/>
       <c r="C63" s="10"/>
@@ -2601,7 +3957,7 @@
       <c r="J63" s="9"/>
       <c r="K63" s="9"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="64" spans="1:11">
       <c r="A64" s="10"/>
       <c r="B64" s="10"/>
       <c r="C64" s="10"/>
@@ -2611,7 +3967,7 @@
       <c r="J64" s="9"/>
       <c r="K64" s="9"/>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="65" spans="1:11">
       <c r="A65" s="10"/>
       <c r="B65" s="10"/>
       <c r="C65" s="10"/>
@@ -2621,7 +3977,7 @@
       <c r="J65" s="9"/>
       <c r="K65" s="9"/>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="66" spans="1:11">
       <c r="A66" s="10"/>
       <c r="B66" s="10"/>
       <c r="C66" s="10"/>
@@ -2631,7 +3987,7 @@
       <c r="J66" s="9"/>
       <c r="K66" s="9"/>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="67" spans="1:11">
       <c r="A67" s="10"/>
       <c r="B67" s="10"/>
       <c r="C67" s="10"/>
@@ -2641,7 +3997,7 @@
       <c r="J67" s="9"/>
       <c r="K67" s="9"/>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="68" spans="1:11">
       <c r="A68" s="10"/>
       <c r="B68" s="10"/>
       <c r="C68" s="10"/>
@@ -2651,7 +4007,7 @@
       <c r="J68" s="9"/>
       <c r="K68" s="9"/>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="69" spans="1:11">
       <c r="A69" s="10"/>
       <c r="B69" s="10"/>
       <c r="C69" s="10"/>
@@ -2661,7 +4017,7 @@
       <c r="J69" s="9"/>
       <c r="K69" s="9"/>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="70" spans="1:11">
       <c r="A70" s="10"/>
       <c r="B70" s="10"/>
       <c r="C70" s="10"/>
@@ -2671,7 +4027,7 @@
       <c r="J70" s="9"/>
       <c r="K70" s="9"/>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="71" spans="1:11">
       <c r="A71" s="10"/>
       <c r="B71" s="10"/>
       <c r="C71" s="10"/>
@@ -2681,7 +4037,7 @@
       <c r="J71" s="9"/>
       <c r="K71" s="9"/>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="72" spans="1:11">
       <c r="A72" s="10"/>
       <c r="B72" s="10"/>
       <c r="C72" s="10"/>
@@ -2691,7 +4047,7 @@
       <c r="J72" s="9"/>
       <c r="K72" s="9"/>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="73" spans="1:11">
       <c r="A73" s="10"/>
       <c r="B73" s="10"/>
       <c r="C73" s="10"/>
@@ -2701,7 +4057,7 @@
       <c r="J73" s="9"/>
       <c r="K73" s="9"/>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="74" spans="1:11">
       <c r="A74" s="10"/>
       <c r="B74" s="10"/>
       <c r="C74" s="10"/>
@@ -2711,7 +4067,7 @@
       <c r="J74" s="9"/>
       <c r="K74" s="9"/>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="75" spans="1:11">
       <c r="A75" s="10"/>
       <c r="B75" s="10"/>
       <c r="C75" s="10"/>
@@ -2721,7 +4077,7 @@
       <c r="J75" s="9"/>
       <c r="K75" s="9"/>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="76" spans="1:11">
       <c r="A76" s="10"/>
       <c r="B76" s="10"/>
       <c r="C76" s="10"/>
@@ -2731,7 +4087,7 @@
       <c r="J76" s="9"/>
       <c r="K76" s="9"/>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="77" spans="1:11">
       <c r="A77" s="10"/>
       <c r="B77" s="10"/>
       <c r="C77" s="10"/>
@@ -2741,7 +4097,7 @@
       <c r="J77" s="9"/>
       <c r="K77" s="9"/>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="78" spans="1:11">
       <c r="A78" s="10"/>
       <c r="B78" s="10"/>
       <c r="C78" s="10"/>
@@ -2751,7 +4107,7 @@
       <c r="J78" s="9"/>
       <c r="K78" s="9"/>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="79" spans="1:11">
       <c r="A79" s="10"/>
       <c r="B79" s="10"/>
       <c r="C79" s="10"/>
@@ -2761,7 +4117,7 @@
       <c r="J79" s="9"/>
       <c r="K79" s="9"/>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="80" spans="1:11">
       <c r="A80" s="10"/>
       <c r="B80" s="10"/>
       <c r="C80" s="10"/>
@@ -2771,7 +4127,7 @@
       <c r="J80" s="9"/>
       <c r="K80" s="9"/>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="81" spans="1:11">
       <c r="A81" s="10"/>
       <c r="B81" s="10"/>
       <c r="C81" s="10"/>
@@ -2781,7 +4137,7 @@
       <c r="J81" s="9"/>
       <c r="K81" s="9"/>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="82" spans="1:11">
       <c r="A82" s="10"/>
       <c r="B82" s="10"/>
       <c r="C82" s="10"/>
@@ -2791,7 +4147,7 @@
       <c r="J82" s="9"/>
       <c r="K82" s="9"/>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="83" spans="1:11">
       <c r="A83" s="10"/>
       <c r="B83" s="10"/>
       <c r="C83" s="10"/>
@@ -2801,7 +4157,7 @@
       <c r="J83" s="9"/>
       <c r="K83" s="9"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="84" spans="1:11">
       <c r="A84" s="10"/>
       <c r="B84" s="10"/>
       <c r="C84" s="10"/>
@@ -2811,7 +4167,7 @@
       <c r="J84" s="9"/>
       <c r="K84" s="9"/>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="85" spans="1:11">
       <c r="A85" s="10"/>
       <c r="B85" s="10"/>
       <c r="C85" s="10"/>
@@ -2821,7 +4177,7 @@
       <c r="J85" s="9"/>
       <c r="K85" s="9"/>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="86" spans="1:11">
       <c r="A86" s="10"/>
       <c r="B86" s="10"/>
       <c r="C86" s="10"/>
@@ -2831,7 +4187,7 @@
       <c r="J86" s="9"/>
       <c r="K86" s="9"/>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="87" spans="1:11">
       <c r="A87" s="10"/>
       <c r="B87" s="10"/>
       <c r="C87" s="10"/>
@@ -2841,7 +4197,7 @@
       <c r="J87" s="9"/>
       <c r="K87" s="9"/>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="88" spans="1:11">
       <c r="A88" s="10"/>
       <c r="B88" s="10"/>
       <c r="C88" s="10"/>
@@ -2851,7 +4207,7 @@
       <c r="J88" s="9"/>
       <c r="K88" s="9"/>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="89" spans="1:11">
       <c r="A89" s="10"/>
       <c r="B89" s="10"/>
       <c r="C89" s="10"/>
@@ -2861,7 +4217,7 @@
       <c r="J89" s="9"/>
       <c r="K89" s="9"/>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="90" spans="1:11">
       <c r="A90" s="10"/>
       <c r="B90" s="10"/>
       <c r="C90" s="10"/>
@@ -2871,7 +4227,7 @@
       <c r="J90" s="9"/>
       <c r="K90" s="9"/>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="91" spans="1:11">
       <c r="A91" s="10"/>
       <c r="B91" s="10"/>
       <c r="C91" s="10"/>
@@ -2881,7 +4237,7 @@
       <c r="J91" s="9"/>
       <c r="K91" s="9"/>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="92" spans="1:11">
       <c r="A92" s="10"/>
       <c r="B92" s="10"/>
       <c r="C92" s="10"/>
@@ -2891,7 +4247,7 @@
       <c r="J92" s="9"/>
       <c r="K92" s="9"/>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="93" spans="1:11">
       <c r="A93" s="10"/>
       <c r="B93" s="10"/>
       <c r="C93" s="10"/>
@@ -2901,7 +4257,7 @@
       <c r="J93" s="9"/>
       <c r="K93" s="9"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="94" spans="1:11">
       <c r="A94" s="10"/>
       <c r="B94" s="10"/>
       <c r="C94" s="10"/>
@@ -2911,7 +4267,7 @@
       <c r="J94" s="9"/>
       <c r="K94" s="9"/>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="95" spans="1:11">
       <c r="A95" s="10"/>
       <c r="B95" s="10"/>
       <c r="C95" s="10"/>
@@ -2921,7 +4277,7 @@
       <c r="J95" s="9"/>
       <c r="K95" s="9"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="96" spans="1:11">
       <c r="A96" s="10"/>
       <c r="B96" s="10"/>
       <c r="C96" s="10"/>
@@ -2931,7 +4287,7 @@
       <c r="J96" s="9"/>
       <c r="K96" s="9"/>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="97" spans="1:11">
       <c r="A97" s="10"/>
       <c r="B97" s="10"/>
       <c r="C97" s="10"/>
@@ -2941,7 +4297,7 @@
       <c r="J97" s="9"/>
       <c r="K97" s="9"/>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="98" spans="1:11">
       <c r="A98" s="10"/>
       <c r="B98" s="10"/>
       <c r="C98" s="10"/>
@@ -2951,7 +4307,7 @@
       <c r="J98" s="9"/>
       <c r="K98" s="9"/>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="99" spans="1:11">
       <c r="A99" s="10"/>
       <c r="B99" s="10"/>
       <c r="C99" s="10"/>
@@ -2961,7 +4317,7 @@
       <c r="J99" s="9"/>
       <c r="K99" s="9"/>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.7">
+    <row r="100" spans="1:11">
       <c r="A100" s="10"/>
       <c r="B100" s="10"/>
       <c r="C100" s="10"/>

</xml_diff>